<commit_message>
Update tour import dialog and agent metadata
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/docs/master-tour-template.xlsx
+++ b/docs/master-tour-template.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -444,17 +444,37 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>7. Imported tours are created as DRAFTS — review, then publish from the Tours page.</v>
+        <v>7. PRICES ARE CALCULATED AUTOMATICALLY by the pricing engine from the services you list here (hotels, guides, sights, transport)</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>8. Upload in Staff Portal → Tours → Import Excel.</v>
+        <v xml:space="preserve">   plus what you configure in the Pricing screens: company margin, free tour-leader policy, group-size bus costing,</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v xml:space="preserve">   airfare per departure city and season, and taxes/fees. You do NOT need to fill any price on the Tours sheet.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>8. basePrice / childPrice / singleSupplement are OPTIONAL fallbacks, shown only while a tour has no pricing data yet. Leave them blank.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>9. Imported tours are created as DRAFTS — review them, set up pricing, then publish from the Tours page.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>10. Upload in Staff Portal → Tours → Import Excel.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A14"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -480,28 +500,28 @@
         <v>countries</v>
       </c>
       <c r="F1" t="str">
+        <v>highlights</v>
+      </c>
+      <c r="G1" t="str">
+        <v>inclusions</v>
+      </c>
+      <c r="H1" t="str">
+        <v>exclusions</v>
+      </c>
+      <c r="I1" t="str">
+        <v>tags</v>
+      </c>
+      <c r="J1" t="str">
+        <v>imageUrl</v>
+      </c>
+      <c r="K1" t="str">
         <v>basePrice</v>
       </c>
-      <c r="G1" t="str">
+      <c r="L1" t="str">
         <v>childPrice</v>
       </c>
-      <c r="H1" t="str">
+      <c r="M1" t="str">
         <v>singleSupplement</v>
-      </c>
-      <c r="I1" t="str">
-        <v>highlights</v>
-      </c>
-      <c r="J1" t="str">
-        <v>inclusions</v>
-      </c>
-      <c r="K1" t="str">
-        <v>exclusions</v>
-      </c>
-      <c r="L1" t="str">
-        <v>tags</v>
-      </c>
-      <c r="M1" t="str">
-        <v>imageUrl</v>
       </c>
     </row>
     <row r="2">
@@ -520,26 +540,26 @@
       <c r="E2" t="str">
         <v>Israel</v>
       </c>
-      <c r="F2">
-        <v>800</v>
-      </c>
-      <c r="G2">
-        <v>400</v>
-      </c>
-      <c r="H2">
-        <v>250</v>
+      <c r="F2" t="str">
+        <v>Old City of Jerusalem; Dead Sea</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Hotels; Guide; Transport</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Flights; Travel insurance</v>
       </c>
       <c r="I2" t="str">
-        <v>Old City of Jerusalem; Dead Sea</v>
+        <v>faith, history</v>
       </c>
       <c r="J2" t="str">
-        <v>Hotels; Guide; Transport</v>
+        <v/>
       </c>
       <c r="K2" t="str">
-        <v>Flights; Travel insurance</v>
+        <v/>
       </c>
       <c r="L2" t="str">
-        <v>faith, history</v>
+        <v/>
       </c>
       <c r="M2" t="str">
         <v/>

</xml_diff>